<commit_message>
fix: BUG #1 — Scenario Manager TypeError crash on Financial page
PROBLEM: json.loads() was called on config_json which could be
either a string (from DB) or already-parsed dict (from database.py
auto-parsing). This caused:
  TypeError: the JSON object must be str, bytes or bytearray, not dict

FIX: Added isinstance() check before json.loads():
  snap = json.loads(raw) if isinstance(raw, str) else (raw if isinstance(raw, dict) else {})

This handles both cases safely — string from DB gets parsed,
dict that's already parsed gets used directly.

VERIFIED: Test confirms no crash with both string and dict inputs.

Also scanned entire codebase — no other json.loads on config_json found.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/auto_synced/Financial_Model_20MT_Uttar_Pradesh.xlsx
+++ b/data/auto_synced/Financial_Model_20MT_Uttar_Pradesh.xlsx
@@ -490,7 +490,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rs 4.80 Crore</t>
+          <t>Rs 4.00 Crore</t>
         </is>
       </c>
     </row>
@@ -502,7 +502,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Rs 3.20 Crore</t>
+          <t>Rs 4.00 Crore</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rs 8.35 Lakhs</t>
+          <t>Rs 7.50 Lakhs</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Rs 13.8 Lakhs</t>
+          <t>Rs 13.7 Lakhs</t>
         </is>
       </c>
     </row>
@@ -610,7 +610,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>20.7%</t>
+          <t>20.6%</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>32.2%</t>
+          <t>26.1%</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1.93x</t>
+          <t>2.14x</t>
         </is>
       </c>
     </row>
@@ -764,22 +764,22 @@
         <v>80</v>
       </c>
       <c r="I2" t="n">
-        <v>55.2</v>
+        <v>56</v>
       </c>
       <c r="J2" t="n">
-        <v>12.4</v>
+        <v>11.6</v>
       </c>
       <c r="K2" t="n">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
       <c r="L2" t="n">
-        <v>9.300000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="M2" t="n">
-        <v>89.3</v>
+        <v>88.7</v>
       </c>
       <c r="N2" t="n">
-        <v>0.89</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="3">
@@ -810,22 +810,22 @@
         <v>80</v>
       </c>
       <c r="I3" t="n">
-        <v>55.2</v>
+        <v>56</v>
       </c>
       <c r="J3" t="n">
-        <v>81.7</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>20.42</v>
+        <v>20.22</v>
       </c>
       <c r="L3" t="n">
-        <v>61.27</v>
+        <v>60.67</v>
       </c>
       <c r="M3" t="n">
-        <v>141.27</v>
+        <v>140.67</v>
       </c>
       <c r="N3" t="n">
-        <v>1.41</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="4">
@@ -856,22 +856,22 @@
         <v>80</v>
       </c>
       <c r="I4" t="n">
-        <v>55.2</v>
+        <v>56</v>
       </c>
       <c r="J4" t="n">
-        <v>151</v>
+        <v>150.2</v>
       </c>
       <c r="K4" t="n">
-        <v>37.75</v>
+        <v>37.55</v>
       </c>
       <c r="L4" t="n">
-        <v>113.25</v>
+        <v>112.65</v>
       </c>
       <c r="M4" t="n">
-        <v>193.25</v>
+        <v>192.65</v>
       </c>
       <c r="N4" t="n">
-        <v>1.93</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="5">
@@ -902,22 +902,22 @@
         <v>80</v>
       </c>
       <c r="I5" t="n">
-        <v>55.2</v>
+        <v>56</v>
       </c>
       <c r="J5" t="n">
-        <v>197.2</v>
+        <v>196.4</v>
       </c>
       <c r="K5" t="n">
-        <v>49.3</v>
+        <v>49.1</v>
       </c>
       <c r="L5" t="n">
-        <v>147.9</v>
+        <v>147.3</v>
       </c>
       <c r="M5" t="n">
-        <v>227.9</v>
+        <v>227.3</v>
       </c>
       <c r="N5" t="n">
-        <v>2.27</v>
+        <v>2.53</v>
       </c>
     </row>
     <row r="6">
@@ -948,22 +948,22 @@
         <v>80</v>
       </c>
       <c r="I6" t="n">
-        <v>55.2</v>
+        <v>56</v>
       </c>
       <c r="J6" t="n">
-        <v>220.3</v>
+        <v>219.5</v>
       </c>
       <c r="K6" t="n">
-        <v>55.08</v>
+        <v>54.88</v>
       </c>
       <c r="L6" t="n">
-        <v>165.23</v>
+        <v>164.63</v>
       </c>
       <c r="M6" t="n">
-        <v>245.23</v>
+        <v>244.63</v>
       </c>
       <c r="N6" t="n">
-        <v>2.45</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="7">
@@ -994,22 +994,22 @@
         <v>80</v>
       </c>
       <c r="I7" t="n">
-        <v>55.2</v>
+        <v>56</v>
       </c>
       <c r="J7" t="n">
-        <v>243.4</v>
+        <v>242.6</v>
       </c>
       <c r="K7" t="n">
-        <v>60.85</v>
+        <v>60.65</v>
       </c>
       <c r="L7" t="n">
-        <v>182.55</v>
+        <v>181.95</v>
       </c>
       <c r="M7" t="n">
-        <v>262.55</v>
+        <v>261.95</v>
       </c>
       <c r="N7" t="n">
-        <v>2.62</v>
+        <v>2.91</v>
       </c>
     </row>
     <row r="8">
@@ -1040,22 +1040,22 @@
         <v>80</v>
       </c>
       <c r="I8" t="n">
-        <v>55.2</v>
+        <v>56</v>
       </c>
       <c r="J8" t="n">
-        <v>243.4</v>
+        <v>242.6</v>
       </c>
       <c r="K8" t="n">
-        <v>60.85</v>
+        <v>60.65</v>
       </c>
       <c r="L8" t="n">
-        <v>182.55</v>
+        <v>181.95</v>
       </c>
       <c r="M8" t="n">
-        <v>262.55</v>
+        <v>261.95</v>
       </c>
       <c r="N8" t="n">
-        <v>2.62</v>
+        <v>2.91</v>
       </c>
     </row>
   </sheetData>
@@ -1365,7 +1365,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>14.0%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">

</xml_diff>